<commit_message>
Adjust column widths in parser_insert_turn.xlsx
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/parser_insert_turn.xlsx
+++ b/parser_insert_turn.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Cursor_progects\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A746A84-DC5E-459D-803C-05CA5FCD325C}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C82663D9-0B2C-427A-91F5-D9760B5643B1}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1980" yWindow="1620" windowWidth="26205" windowHeight="13320" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -337,12 +337,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -358,12 +364,16 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -66767,15 +66777,21 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.125" customWidth="1"/>
-    <col min="3" max="3" width="5" customWidth="1"/>
-    <col min="6" max="6" width="28.875" customWidth="1"/>
+    <col min="2" max="2" width="9" style="5"/>
+    <col min="3" max="3" width="3.625" style="4" customWidth="1"/>
+    <col min="5" max="5" width="40" customWidth="1"/>
+    <col min="6" max="6" width="3.625" style="4" customWidth="1"/>
+    <col min="8" max="8" width="16.625" customWidth="1"/>
+    <col min="9" max="9" width="3.625" style="4" customWidth="1"/>
+    <col min="14" max="14" width="3.625" style="4" customWidth="1"/>
+    <col min="16" max="16" width="50.75" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="5" t="s">
         <v>4</v>
       </c>
       <c r="D1" t="s">
@@ -66813,7 +66829,7 @@
       <c r="A2" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="5" t="s">
         <v>21</v>
       </c>
       <c r="D2" t="s">
@@ -66851,7 +66867,7 @@
       <c r="A3" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="5" t="s">
         <v>32</v>
       </c>
       <c r="D3" t="s">
@@ -66883,7 +66899,7 @@
       <c r="A4" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B4" s="5" t="s">
         <v>39</v>
       </c>
       <c r="D4" t="s">
@@ -66915,7 +66931,7 @@
       <c r="A5" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B5" s="5" t="s">
         <v>46</v>
       </c>
       <c r="D5" t="s">
@@ -66947,7 +66963,7 @@
       <c r="A6" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="B6" t="s">
+      <c r="B6" s="5" t="s">
         <v>53</v>
       </c>
       <c r="D6" t="s">
@@ -66979,7 +66995,7 @@
       <c r="A7" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="B7" t="s">
+      <c r="B7" s="5" t="s">
         <v>60</v>
       </c>
       <c r="D7" t="s">
@@ -67011,7 +67027,7 @@
       <c r="A8" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="B8" t="s">
+      <c r="B8" s="5" t="s">
         <v>67</v>
       </c>
       <c r="D8" t="s">
@@ -67037,7 +67053,7 @@
       <c r="A9" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="B9" t="s">
+      <c r="B9" s="5" t="s">
         <v>71</v>
       </c>
       <c r="D9" t="s">
@@ -67057,7 +67073,7 @@
       <c r="A10" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="B10">
+      <c r="B10" s="5">
         <v>11.11</v>
       </c>
       <c r="D10" t="s">
@@ -67071,7 +67087,7 @@
       <c r="A11" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="B11">
+      <c r="B11" s="5">
         <v>12.7</v>
       </c>
       <c r="D11" t="s">
@@ -67085,7 +67101,7 @@
       <c r="A12" t="s">
         <v>91</v>
       </c>
-      <c r="B12">
+      <c r="B12" s="5">
         <v>1.98</v>
       </c>
       <c r="D12" t="s">
@@ -67099,7 +67115,7 @@
       <c r="A13" s="3" t="s">
         <v>92</v>
       </c>
-      <c r="B13">
+      <c r="B13" s="5">
         <v>2.78</v>
       </c>
       <c r="D13" t="s">
@@ -67113,7 +67129,7 @@
       <c r="A14" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="B14">
+      <c r="B14" s="5">
         <v>3.97</v>
       </c>
       <c r="D14" t="s">

</xml_diff>

<commit_message>
Keep leading zeros in re lookup codes on Map sheet
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/parser_insert_turn.xlsx
+++ b/parser_insert_turn.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Cursor_progects\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FDB1A22C-9A07-456E-91E0-D1A8DF0DBA85}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC50786D-F09A-49A6-A65A-27ED2DE55DDC}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1980" yWindow="1620" windowWidth="26205" windowHeight="13320" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="139" uniqueCount="98">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="105">
   <si>
     <t>art</t>
   </si>
@@ -323,6 +323,27 @@
   </si>
   <si>
     <t>M0</t>
+  </si>
+  <si>
+    <t>08</t>
+  </si>
+  <si>
+    <t>16</t>
+  </si>
+  <si>
+    <t>20</t>
+  </si>
+  <si>
+    <t>24</t>
+  </si>
+  <si>
+    <t>28</t>
+  </si>
+  <si>
+    <t>32</t>
+  </si>
+  <si>
+    <t>00</t>
   </si>
 </sst>
 </file>
@@ -773,9 +794,9 @@
         <f>IFERROR(VLOOKUP(MID(A2,7,2),Map!$A$2:$B$20,2,FALSE),"")</f>
         <v>3.97</v>
       </c>
-      <c r="F2" t="str">
+      <c r="F2">
         <f>IF(A2="","",IFERROR(VLOOKUP(MID(A2,9,2),Map!$R$2:$S$14,2,FALSE),""))</f>
-        <v/>
+        <v>0.8</v>
       </c>
       <c r="G2" t="str">
         <f t="shared" ref="G2:G65" si="3">IFERROR(MID(A2,FIND("-",A2)+1,FIND("-",A2,FIND("-",A2)+1)-FIND("-",A2)-1),"")</f>
@@ -842,9 +863,9 @@
         <f>IFERROR(VLOOKUP(MID(A3,7,2),Map!$A$2:$B$20,2,FALSE),"")</f>
         <v>3.18</v>
       </c>
-      <c r="F3" t="str">
+      <c r="F3">
         <f>IF(A3="","",IFERROR(VLOOKUP(MID(A3,9,2),Map!$R$2:$S$14,2,FALSE),""))</f>
-        <v/>
+        <v>0.8</v>
       </c>
       <c r="G3" t="str">
         <f t="shared" si="3"/>
@@ -911,9 +932,9 @@
         <f>IFERROR(VLOOKUP(MID(A4,7,2),Map!$A$2:$B$20,2,FALSE),"")</f>
         <v/>
       </c>
-      <c r="F4" t="str">
+      <c r="F4">
         <f>IF(A4="","",IFERROR(VLOOKUP(MID(A4,9,2),Map!$R$2:$S$14,2,FALSE),""))</f>
-        <v/>
+        <v>0.8</v>
       </c>
       <c r="G4" t="str">
         <f t="shared" si="3"/>
@@ -980,9 +1001,9 @@
         <f>IFERROR(VLOOKUP(MID(A5,7,2),Map!$A$2:$B$20,2,FALSE),"")</f>
         <v>4.76</v>
       </c>
-      <c r="F5" t="str">
+      <c r="F5">
         <f>IF(A5="","",IFERROR(VLOOKUP(MID(A5,9,2),Map!$R$2:$S$14,2,FALSE),""))</f>
-        <v/>
+        <v>0.4</v>
       </c>
       <c r="G5" t="str">
         <f t="shared" si="3"/>
@@ -1049,9 +1070,9 @@
         <f>IFERROR(VLOOKUP(MID(A6,7,2),Map!$A$2:$B$20,2,FALSE),"")</f>
         <v>4.76</v>
       </c>
-      <c r="F6" t="str">
+      <c r="F6">
         <f>IF(A6="","",IFERROR(VLOOKUP(MID(A6,9,2),Map!$R$2:$S$14,2,FALSE),""))</f>
-        <v/>
+        <v>0.4</v>
       </c>
       <c r="G6" t="str">
         <f t="shared" si="3"/>
@@ -66794,6 +66815,7 @@
     <col min="9" max="9" width="3.625" style="4" customWidth="1"/>
     <col min="14" max="14" width="3.625" style="4" customWidth="1"/>
     <col min="16" max="16" width="50.75" customWidth="1"/>
+    <col min="18" max="18" width="9" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:19" x14ac:dyDescent="0.25">
@@ -66833,7 +66855,7 @@
       <c r="P1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="1" t="s">
         <v>19</v>
       </c>
       <c r="S1" t="s">
@@ -66877,7 +66899,7 @@
       <c r="P2" t="s">
         <v>30</v>
       </c>
-      <c r="R2" t="s">
+      <c r="R2" s="1" t="s">
         <v>95</v>
       </c>
       <c r="S2">
@@ -66915,8 +66937,8 @@
       <c r="P3" t="s">
         <v>37</v>
       </c>
-      <c r="R3">
-        <v>1</v>
+      <c r="R3" s="1" t="s">
+        <v>20</v>
       </c>
       <c r="S3">
         <v>0.1</v>
@@ -66953,8 +66975,8 @@
       <c r="P4" t="s">
         <v>44</v>
       </c>
-      <c r="R4">
-        <v>2</v>
+      <c r="R4" s="1" t="s">
+        <v>31</v>
       </c>
       <c r="S4">
         <v>0.2</v>
@@ -66991,8 +67013,8 @@
       <c r="P5" t="s">
         <v>51</v>
       </c>
-      <c r="R5">
-        <v>4</v>
+      <c r="R5" s="1" t="s">
+        <v>45</v>
       </c>
       <c r="S5">
         <v>0.4</v>
@@ -67029,8 +67051,8 @@
       <c r="P6" t="s">
         <v>58</v>
       </c>
-      <c r="R6">
-        <v>8</v>
+      <c r="R6" s="1" t="s">
+        <v>98</v>
       </c>
       <c r="S6">
         <v>0.8</v>
@@ -67067,8 +67089,8 @@
       <c r="P7" t="s">
         <v>65</v>
       </c>
-      <c r="R7">
-        <v>12</v>
+      <c r="R7" s="1" t="s">
+        <v>78</v>
       </c>
       <c r="S7">
         <v>1.2</v>
@@ -67099,8 +67121,8 @@
       <c r="P8" t="s">
         <v>69</v>
       </c>
-      <c r="R8">
-        <v>16</v>
+      <c r="R8" s="1" t="s">
+        <v>99</v>
       </c>
       <c r="S8">
         <v>1.6</v>
@@ -67125,8 +67147,8 @@
       <c r="P9" t="s">
         <v>74</v>
       </c>
-      <c r="R9">
-        <v>20</v>
+      <c r="R9" s="1" t="s">
+        <v>100</v>
       </c>
       <c r="S9">
         <v>2</v>
@@ -67145,8 +67167,8 @@
       <c r="E10" t="s">
         <v>77</v>
       </c>
-      <c r="R10">
-        <v>24</v>
+      <c r="R10" s="1" t="s">
+        <v>101</v>
       </c>
       <c r="S10">
         <v>2.4</v>
@@ -67165,8 +67187,8 @@
       <c r="E11" t="s">
         <v>79</v>
       </c>
-      <c r="R11">
-        <v>28</v>
+      <c r="R11" s="1" t="s">
+        <v>102</v>
       </c>
       <c r="S11">
         <v>2.8</v>
@@ -67185,8 +67207,8 @@
       <c r="E12" t="s">
         <v>80</v>
       </c>
-      <c r="R12">
-        <v>32</v>
+      <c r="R12" s="1" t="s">
+        <v>103</v>
       </c>
       <c r="S12">
         <v>3.2</v>
@@ -67205,8 +67227,8 @@
       <c r="E13" t="s">
         <v>81</v>
       </c>
-      <c r="R13">
-        <v>0</v>
+      <c r="R13" s="1" t="s">
+        <v>104</v>
       </c>
       <c r="S13" t="s">
         <v>96</v>
@@ -67225,7 +67247,7 @@
       <c r="E14" t="s">
         <v>83</v>
       </c>
-      <c r="R14" t="s">
+      <c r="R14" s="1" t="s">
         <v>97</v>
       </c>
       <c r="S14" t="s">

</xml_diff>